<commit_message>
feat: update speaker session room names for consistency and clarity; adjust navbar positioning for talk schedule
</commit_message>
<xml_diff>
--- a/src/assets/speakers/data-advanced.xlsx
+++ b/src/assets/speakers/data-advanced.xlsx
@@ -220,7 +220,7 @@
     <t>DevOps</t>
   </si>
   <si>
-    <t>Sala Fibonacci (35 posti)</t>
+    <t>Sala Fibonacci</t>
   </si>
   <si>
     <t>28b496fc-f417-409d-a957-b79e59aca43c</t>
@@ -247,7 +247,7 @@
     <t>Germany</t>
   </si>
   <si>
-    <t>Sala Ricci (150 posti)</t>
+    <t>Sala Ricci</t>
   </si>
   <si>
     <t>d7da8026-334b-42d8-aec9-324bf1bb6ec4</t>
@@ -278,7 +278,7 @@
     <t>United Kingdom</t>
   </si>
   <si>
-    <t>Sala Gentili (35 posti) Build with AI</t>
+    <t>Sala Gentili Build with AI</t>
   </si>
   <si>
     <t>fec11d0b-9f52-4f13-8c44-a4afe2b76204</t>
@@ -304,7 +304,7 @@
     <t>Pietro Tempesti, Franco Riformato</t>
   </si>
   <si>
-    <t>Sala Pacinotti (50 posti)</t>
+    <t>Sala Pacinotti</t>
   </si>
   <si>
     <t>3b452ac7-f8a5-426f-ac8b-6d5439967ef5, 62596635-c196-410f-badd-412acdebfb95</t>

</xml_diff>